<commit_message>
baselines: trim each to its scanner's own columns
The union layout left every baseline carrying foreign, always-empty columns
(e.g. instances on OpenVAS). trim_baseline_columns.py drops them so each
baseline matches its scanner's record model, which is also cleaner as a
dataset. Lossless: only empty columns are removed. Nessus baselines were
already generated trimmed.
</commit_message>
<xml_diff>
--- a/resources/openvas/OpenVAS_JuiceShop.xlsx
+++ b/resources/openvas/OpenVAS_JuiceShop.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S35"/>
+  <dimension ref="A1:P35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -497,21 +497,6 @@
           <t>log_method</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>plugin</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>plugin_details</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>instances</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -529,14 +514,11 @@
           <t>Contact the vendor of the antivirus scanner to get an update.</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
         <v>25</v>
       </c>
@@ -553,7 +535,6 @@
       <c r="K2" t="n">
         <v>7.5</v>
       </c>
-      <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
           <t>Vulnerability was detected according to the Vulnerability Detection Method.</t>
@@ -562,19 +543,6 @@
       <c r="N2" t="inlineStr">
         <is>
           <t>Details: SMTP too long line OID:1.3.6.1.4.1.25623.1.0.11270 Version used: $Revision: 13470 $</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>[]</t>
         </is>
       </c>
     </row>
@@ -599,13 +567,11 @@
           <t>This issue may be exploited by a remote attacker to gain access to sensitive information or modify system configuration.</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
         <v>9390</v>
       </c>
@@ -642,18 +608,6 @@
           <t>Product: cpe:/a:openvas:openvas_manager:7.0 Method: OpenVAS / Greenbone Vulnerability Manager Detection OID: 1.3.6.1.4.1.25623.1.0.103825</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -671,14 +625,11 @@
           <t>Replace the SSL/TLS certicate by a new one.</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
         <v>443</v>
       </c>
@@ -722,19 +673,6 @@
           <t>Details: SSL/TLS: Certificate Expired OID:1.3.6.1.4.1.25623.1.0.103955 Version used: $Revision: 11103 $</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -752,7 +690,6 @@
           <t>Disable VRFY and/or EXPN on your Mailserver.</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>['URL:http://cr.yp.to/smtp/vrfy.html']</t>
@@ -763,7 +700,6 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
         <v>25</v>
       </c>
@@ -795,19 +731,6 @@
           <t>Details: Check if Mailserver answer to VRFY and EXPN requests OID:1.3.6.1.4.1.25623.1.0.100072 Version used: $Revision: 13470 $</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -825,14 +748,11 @@
           <t>Replace the SSL/TLS certicate by a new one.</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
         <v>9390</v>
       </c>
@@ -876,19 +796,6 @@
           <t>Details: SSL/TLS: Certificate Expired OID:1.3.6.1.4.1.25623.1.0.103955 Version used: $Revision: 11103 $</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -911,8 +818,6 @@
 If you think any of this information is wrong please report it to the referenced community portal.</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>['URL:https://community.greenbone.net/c/vulnerability-tests']</t>
@@ -923,7 +828,6 @@
           <t>LOG</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
         <v>443</v>
       </c>
@@ -940,7 +844,6 @@
       <c r="K7" t="n">
         <v>0</v>
       </c>
-      <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
           <t>The Hostname/IP "localhost" was used to access the remote host.
@@ -973,22 +876,9 @@
 https://localhost/omp (cmd [login] text [/omp?r=1] login [] password [] )</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
           <t>Details: CGI Scanning Consolidation OID:1.3.6.1.4.1.25623.1.0.111038 Version used: $Revision: 13679 $</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>[]</t>
         </is>
       </c>
     </row>
@@ -1003,15 +893,11 @@
           <t>The script sends a connection request to the server and attempts to determine if it is a GSA from the reply.</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>LOG</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
         <v>443</v>
       </c>
@@ -1028,7 +914,6 @@
       <c r="K8" t="n">
         <v>0</v>
       </c>
-      <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
           <t>Detected Greenbone Security Assistant
@@ -1039,22 +924,9 @@
 Version 7.0.3</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
         <is>
           <t>Details: Greenbone Security Assistant (GSA) Detection OID:1.3.6.1.4.1.25623.1.0.103841 Version used: $Revision: 13882 $</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>[]</t>
         </is>
       </c>
     </row>
@@ -1071,8 +943,6 @@
 on the target.</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>['URL:https://www.owasp.org/index.php/OWASP_Secure_Headers_Project', 'URL:https://www.owasp.org/index.php/OWASP_Secure_Headers_Project#tab=Headers', 'URL:https://securityheaders.io/']</t>
@@ -1083,7 +953,6 @@
           <t>LOG</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
         <v>443</v>
       </c>
@@ -1100,7 +969,6 @@
       <c r="K9" t="n">
         <v>0</v>
       </c>
-      <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr">
         <is>
           <t>Header Name Header Value
@@ -1116,22 +984,9 @@
 X-XSS-Protection</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr">
         <is>
           <t>Details: HTTP Security Headers Detection OID:1.3.6.1.4.1.25623.1.0.112081 Version used: $Revision: 10899 $</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>[]</t>
         </is>
       </c>
     </row>
@@ -1148,15 +1003,11 @@
 information available for other check routines.</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>LOG</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
         <v>443</v>
       </c>
@@ -1173,28 +1024,14 @@
       <c r="K10" t="n">
         <v>0</v>
       </c>
-      <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr">
         <is>
           <t>A TLScustom server answered on this port</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr">
         <is>
           <t>Details: Services OID:1.3.6.1.4.1.25623.1.0.10330 Version used: $Revision: 13541 $</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>[]</t>
         </is>
       </c>
     </row>
@@ -1211,15 +1048,11 @@
 information available for other check routines.</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>LOG</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
         <v>443</v>
       </c>
@@ -1236,28 +1069,14 @@
       <c r="K11" t="n">
         <v>0</v>
       </c>
-      <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr">
         <is>
           <t>A web server is running on this port through SSL</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr">
         <is>
           <t>Details: Services OID:1.3.6.1.4.1.25623.1.0.10330 Version used: $Revision: 13541 $</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>[]</t>
         </is>
       </c>
     </row>
@@ -1272,15 +1091,11 @@
           <t>This script collects and reports the details of all SSL/TLS certicates.</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>LOG</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
         <v>443</v>
       </c>
@@ -1297,7 +1112,6 @@
       <c r="K12" t="n">
         <v>0</v>
       </c>
-      <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr">
         <is>
           <t>The following certificate details of the remote service were collected.
@@ -1315,22 +1129,9 @@
 ,!41BC4B9</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr">
         <is>
           <t>Details: SSL/TLS: Collect and Report Certificate Details OID:1.3.6.1.4.1.25623.1.0.103692 Version used: $Revision: 13434 $</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S12" t="inlineStr">
-        <is>
-          <t>[]</t>
         </is>
       </c>
     </row>
@@ -1350,7 +1151,6 @@
           <t>['Enable HPKP or add / congure the required directives correctly following the guides linked in the references.']</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>['URL:https://www.owasp.org/index.php/OWASP_Secure_Headers_Project', 'URL:https://www.owasp.org/index.php/OWASP_Secure_Headers_Project#hpkp', 'URL:https://tools.ietf.org/html/rfc7469', 'URL:https://securityheaders.io/']</t>
@@ -1361,7 +1161,6 @@
           <t>LOG</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
         <v>443</v>
       </c>
@@ -1378,7 +1177,6 @@
       <c r="K13" t="n">
         <v>0</v>
       </c>
-      <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr">
         <is>
           <t>The remote web server is not enforcing HPKP.
@@ -1395,22 +1193,9 @@
 Date: ***replaced***</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr">
         <is>
           <t>Details: SSL/TLS: HTTP Public Key Pinning (HPKP) Missing OID:1.3.6.1.4.1.25623.1.0.108247 Version used: $Revision: 7391 $</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>[]</t>
         </is>
       </c>
     </row>
@@ -1430,7 +1215,6 @@
           <t>Enable HSTS or add / congure the required directives correctly following the guides linked in the references.</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
           <t>['URL:https://www.owasp.org/index.php/OWASP_Secure_Headers_Project', 'URL:https://www.owasp.org/index.php/HTTP_Strict_Transport_Security_Cheat_Sheet', 'URL:https://www.owasp.org/index.php/OWASP_Secure_Headers_Project#hsts', 'URL:https://tools.ietf.org/html/rfc6797', 'URL:https://securityheaders.io/']</t>
@@ -1441,7 +1225,6 @@
           <t>LOG</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
         <v>443</v>
       </c>
@@ -1458,7 +1241,6 @@
       <c r="K14" t="n">
         <v>0</v>
       </c>
-      <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr">
         <is>
           <t>The remote web server is not enforcing HSTS.
@@ -1475,22 +1257,9 @@
 Date: ***replaced***</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr">
         <is>
           <t>Details: SSL/TLS: HTTP Strict Transport Security (HSTS) Missing OID:1.3.6.1.4.1.25623.1.0.105879 Version used: $Revision: 7391 $</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S14" t="inlineStr">
-        <is>
-          <t>[]</t>
         </is>
       </c>
     </row>
@@ -1505,15 +1274,11 @@
           <t>The remote service is missing support for SSL/TLS cipher suites supporting Perfect Forward Secrecy.</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>LOG</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
         <v>443</v>
       </c>
@@ -1530,28 +1295,14 @@
       <c r="K15" t="n">
         <v>0</v>
       </c>
-      <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr">
         <is>
           <t>The remote service does not support perfect forward secrecy cipher suites.</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr">
         <is>
           <t>Details: SSL/TLS: Perfect Forward Secrecy Cipher Suites Missing OID:1.3.6.1.4.1.25623.1.0.105092 Version used: $Revision: 4736 $</t>
-        </is>
-      </c>
-      <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S15" t="inlineStr">
-        <is>
-          <t>[]</t>
         </is>
       </c>
     </row>
@@ -1566,15 +1317,11 @@
           <t>This routine reports all Medium SSL/TLS cipher suites accepted by a service.</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>LOG</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
         <v>443</v>
       </c>
@@ -1614,8 +1361,6 @@
 TLS_RSA_WITH_CAMELLIA_256_GCM_SHA384</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr">
         <is>
           <t>Details: SSL/TLS: Report Medium Cipher Suites
@@ -1623,17 +1368,6 @@
 Version used: $Revision: 4743 $</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S16" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1646,15 +1380,11 @@
           <t>This routine reports all Non Weak SSL/TLS cipher suites accepted by a service.</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>LOG</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
         <v>443</v>
       </c>
@@ -1671,7 +1401,6 @@
       <c r="K17" t="n">
         <v>0</v>
       </c>
-      <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr">
         <is>
           <t>Non Weak' cipher suites accepted by this service via the TLSv1.1 protocol:
@@ -1690,24 +1419,11 @@
 TLS_RSA_WITH_CAMELLIA_256_GCM_SHA384</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr">
         <is>
           <t>Details: SSL/TLS: Report Non Weak Cipher Suites
 OID:1.3.6.1.4.1.25623.1.0.103441
 Version used: $Revision: 4736 $</t>
-        </is>
-      </c>
-      <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S17" t="inlineStr">
-        <is>
-          <t>[]</t>
         </is>
       </c>
     </row>
@@ -1726,15 +1442,11 @@
 is reported.</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
           <t>LOG</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
         <v>443</v>
       </c>
@@ -1751,7 +1463,6 @@
       <c r="K18" t="n">
         <v>0</v>
       </c>
-      <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr">
         <is>
           <t>No 'Strong' cipher suites accepted by this service via the TLSv1.1 protocol. 'Medium' cipher suites accepted by this service via the TLSv1.1 protocol: TLS_RSA_WITH_AES_256_CBC_SHA, TLS_RSA_WITH_CAMELLIA_256_CBC_SHA -TLS_RSA_WITH_CAMELLIA_256_CBC_SHA
@@ -1775,24 +1486,11 @@
 No 'Anonymous' cipher suites accepted by this service via the TLSv1.2 protocol.</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr">
         <is>
           <t>Details: SSL/TLS: Report Supported Cipher Suites
 OID:1.3.6.1.4.1.25623.1.0.802067
 Version used: $Revision: 11108 $</t>
-        </is>
-      </c>
-      <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S18" t="inlineStr">
-        <is>
-          <t>[]</t>
         </is>
       </c>
     </row>
@@ -1814,15 +1512,11 @@
 separately within 'Availability of scanner helper tools' (OID: 1.3.6.1.4.1.25623.1.0.810000).</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
           <t>LOG</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
         <v>443</v>
       </c>
@@ -1839,7 +1533,6 @@
       <c r="K19" t="n">
         <v>0</v>
       </c>
-      <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr">
         <is>
           <t>The wapiti report filename is empty. That could mean that a wrong version of wap
@@ -1848,25 +1541,12 @@
 In short: Check the installation of wapiti and the scanner.</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr">
         <is>
           <t>Details: wapiti (NASL wrapper)
 OID:1.3.6.1.4.1.25623.1.0.80110 Version used: $Revision: 13985 $</t>
         </is>
       </c>
-      <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S19" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1879,15 +1559,11 @@
           <t>The script checks the SMTP server banner for the presence of Postx.</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>LOG</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
         <v>25</v>
       </c>
@@ -1904,7 +1580,6 @@
       <c r="K20" t="n">
         <v>0</v>
       </c>
-      <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr">
         <is>
           <t>Detected Postfix
@@ -1915,8 +1590,6 @@
 220 9c89ef55d1a6.localdomain ESMTP Postfix</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr">
         <is>
           <t>Details: Postfix SMTP Server Detection
@@ -1924,17 +1597,6 @@
 Version used: $Revision: 13461 $</t>
         </is>
       </c>
-      <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S20" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1949,15 +1611,11 @@
 information available for other check routines.</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>LOG</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
         <v>25</v>
       </c>
@@ -1971,15 +1629,11 @@
           <t>OPENVAS</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr">
         <is>
           <t>An SMTP server is running on this port, Here is its banner: 220 9c89ef55d1a6.localdomain ESMTP Postfix</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr">
         <is>
           <t>Details: Services
@@ -1987,17 +1641,6 @@
 Version used: $Revision: 13541 $</t>
         </is>
       </c>
-      <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2015,7 +1658,6 @@
           <t>Reconfigure your antivirus / upgrade it.</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
           <t>['BID:3027']</t>
@@ -2026,7 +1668,6 @@
           <t>LOG</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
         <v>25</v>
       </c>
@@ -2043,7 +1684,6 @@
       <c r="K22" t="n">
         <v>7.2</v>
       </c>
-      <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr">
         <is>
           <t>For some reason, we could not send the 42.zip file to this MTA.</t>
@@ -2056,19 +1696,6 @@
 Version used: $Revision: 13470 $</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2081,15 +1708,11 @@
           <t>The remote SMTP server does not support the 'STARTTLS' command.</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>LOG</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
         <v>25</v>
       </c>
@@ -2106,14 +1729,11 @@
       <c r="K23" t="n">
         <v>0</v>
       </c>
-      <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr">
         <is>
           <t>The remote SMTP server does not support the 'STARTTLS' command.</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr">
         <is>
           <t>Details: SMTP Missing Support For STARTTLS
@@ -2121,17 +1741,6 @@
 Version used: $Revision: 13153 $</t>
         </is>
       </c>
-      <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2144,15 +1753,11 @@
           <t>This detects the SMTP Server's type and version by connecting to the server and processing the buffer received.</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>LOG</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
         <v>25</v>
       </c>
@@ -2169,7 +1774,6 @@
       <c r="K24" t="n">
         <v>0</v>
       </c>
-      <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr">
         <is>
           <t>Remote SMTP server banner: 220 9c89ef55d1a6.localdomain ESMTP Postfix The remote SMTP server is announcing the following available ESMTP commands (EHL
@@ -2177,8 +1781,6 @@
 8BITMIME, DSN, ENHANCEDSTATUSCODES, ETRN, PIPELINING, SIZE 10240000, VRFY</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr">
         <is>
           <t>Details: SMTP Server type and version
@@ -2186,17 +1788,6 @@
 Version used: $Revision: 14004 $</t>
         </is>
       </c>
-      <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S24" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2209,15 +1800,11 @@
           <t>The script sends a connection request to the server and attempts to determine if it is a OpenVAS Manager (openvasmd) or Greenbone Vulnerability Manager (gmvd).</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>LOG</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
       <c r="H25" t="n">
         <v>9390</v>
       </c>
@@ -2234,7 +1821,6 @@
       <c r="K25" t="n">
         <v>0</v>
       </c>
-      <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr">
         <is>
           <t>Detected OpenVAS Manager
@@ -2245,8 +1831,6 @@
 OMP protocol version request '&lt;GET_VERSION/&gt;', response: &lt;version&gt;7.0&lt;/version&gt;</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr">
         <is>
           <t>Details: OpenVAS / Greenbone Vulnerability Manager Detection
@@ -2254,17 +1838,6 @@
 Version used: $Revision: 13874 $</t>
         </is>
       </c>
-      <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S25" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2279,15 +1852,11 @@
 information available for other check routines.</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>LOG</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="n">
         <v>9390</v>
       </c>
@@ -2304,14 +1873,11 @@
       <c r="K26" t="n">
         <v>0</v>
       </c>
-      <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr">
         <is>
           <t>A TLScustom server answered on this port</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr">
         <is>
           <t>Details: Services
@@ -2319,17 +1885,6 @@
 Version used: $Revision: 13541 $</t>
         </is>
       </c>
-      <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S26" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2344,15 +1899,11 @@
 unknown services and tries to identify them.</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>LOG</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
       <c r="H27" t="n">
         <v>9390</v>
       </c>
@@ -2369,14 +1920,11 @@
       <c r="K27" t="n">
         <v>0</v>
       </c>
-      <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr">
         <is>
           <t>A OpenVAS / Greenbone Vulnerability Manager supporting the OMP/GMP protocol seems to be running on this port.</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr">
         <is>
           <t>Details: Service Detection with '&lt;xml/&gt;' Request
@@ -2384,17 +1932,6 @@
 Version used: $Revision: 13874 $</t>
         </is>
       </c>
-      <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S27" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2407,15 +1944,11 @@
           <t>This script collects and reports the details of all SSL/TLS certificates.</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>LOG</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
       <c r="H28" t="n">
         <v>9390</v>
       </c>
@@ -2432,7 +1965,6 @@
       <c r="K28" t="n">
         <v>0</v>
       </c>
-      <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr">
         <is>
           <t>The following certificate details of the remote service were collected.
@@ -2450,22 +1982,9 @@
 ,!41BC4B9</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr">
         <is>
           <t>Details: SSL/TLS: Collect and Report Certificate Details OID:1.3.6.1.4.1.25623.1.0.103692 Version used: $Revision: 13434 $</t>
-        </is>
-      </c>
-      <c r="Q28" t="inlineStr"/>
-      <c r="R28" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S28" t="inlineStr">
-        <is>
-          <t>[]</t>
         </is>
       </c>
     </row>
@@ -2480,15 +1999,11 @@
           <t>The remote service is missing support for SSL/TLS cipher suites supporting Perfect Forward Secrecy.</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>LOG</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
       <c r="H29" t="n">
         <v>9390</v>
       </c>
@@ -2505,14 +2020,11 @@
       <c r="K29" t="n">
         <v>0</v>
       </c>
-      <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr">
         <is>
           <t>The remote service does not support perfect forward secrecy cipher suites.</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr">
         <is>
           <t>Details: SSL/TLS: Perfect Forward Secrecy Cipher Suites Missing
@@ -2520,17 +2032,6 @@
 Version used: $Revision: 4736 $</t>
         </is>
       </c>
-      <c r="Q29" t="inlineStr"/>
-      <c r="R29" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S29" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2543,15 +2044,11 @@
           <t>This routine reports all Medium SSL/TLS cipher suites accepted by a service.</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
           <t>LOG</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
       <c r="H30" t="n">
         <v>9390</v>
       </c>
@@ -2605,8 +2102,6 @@
 TLS_RSA_WITH_CAMELLIA_256_GCM_SHA384</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr">
         <is>
           <t>Details: SSL/TLS: Report Medium Cipher Suites
@@ -2614,17 +2109,6 @@
 Version used: $Revision: 4743 $</t>
         </is>
       </c>
-      <c r="Q30" t="inlineStr"/>
-      <c r="R30" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S30" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2637,15 +2121,11 @@
           <t>This routine reports all Non Weak SSL/TLS cipher suites accepted by a service.</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
           <t>LOG</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
           <t xml:space="preserve">9,390
@@ -2665,7 +2145,6 @@
       <c r="K31" t="n">
         <v>0</v>
       </c>
-      <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr">
         <is>
           <t>Non Weak' cipher suites accepted by this service via the TLSv1.0 protocol:
@@ -2698,24 +2177,11 @@
 TLS_RSA_WITH_CAMELLIA_256_GCM_SHA384</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr">
         <is>
           <t>Details: SSL/TLS: Report Non Weak Cipher Suites
 OID:1.3.6.1.4.1.25623.1.0.103441
 Version used: $Revision: 4736 $</t>
-        </is>
-      </c>
-      <c r="Q31" t="inlineStr"/>
-      <c r="R31" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S31" t="inlineStr">
-        <is>
-          <t>[]</t>
         </is>
       </c>
     </row>
@@ -2734,15 +2200,11 @@
 is reported.</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
           <t>LOG</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
           <t xml:space="preserve">9,390
@@ -2762,7 +2224,6 @@
       <c r="K32" t="n">
         <v>0</v>
       </c>
-      <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr">
         <is>
           <t>No 'Strong' cipher suites accepted by this service via the TLSv1.0 protocol.
@@ -2807,8 +2268,6 @@
 No 'Anonymous' cipher suites accepted by this service via the TLSv1.2 protocol.</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr">
         <is>
           <t>Details: SSL/TLS: Report Supported Cipher Suites
@@ -2816,17 +2275,6 @@
 Version used: $Revision: 11108 $</t>
         </is>
       </c>
-      <c r="Q32" t="inlineStr"/>
-      <c r="R32" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S32" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2839,8 +2287,6 @@
           <t>This routine uses information collected by other routines about CPE identities of operating systems, services and applications detected during the scan.</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
           <t>['http://cpe.mitre.org/']</t>
@@ -2851,7 +2297,6 @@
           <t>LOG</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
           <t>general</t>
@@ -2870,30 +2315,16 @@
       <c r="K33" t="n">
         <v>0</v>
       </c>
-      <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr">
         <is>
           <t>127.0.0.1|cpe:/a:greenbone:greenbone_security_assistant:7.0.3, 127.0.0.1|cpe:/a:openvas:openvas_manager:7.0, 127.0.0.1|cpe:/a:postfix:postfix, 127.0.0.1|cpe:/o:linux:linux_kernel:2.6.32</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr">
         <is>
           <t>Details: CPE Inventory
 OID:1.3.6.1.4.1.25623.1.0.810002
 Version used: $Revision: 14324 $</t>
-        </is>
-      </c>
-      <c r="Q33" t="inlineStr"/>
-      <c r="R33" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S33" t="inlineStr">
-        <is>
-          <t>[]</t>
         </is>
       </c>
     </row>
@@ -2913,8 +2344,6 @@
 referenced community portal.</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
           <t>['https://community.greenbone.net/c/vulnerability-tests']</t>
@@ -2925,7 +2354,6 @@
           <t>LOG</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
           <t>general</t>
@@ -2944,7 +2372,6 @@
       <c r="K34" t="n">
         <v>0</v>
       </c>
-      <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr">
         <is>
           <t>Best matching OS:
@@ -2963,24 +2390,11 @@
 Concluded from ICMP based OS fingerprint</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr">
         <is>
           <t>Details: OS Detection Consolidation and Reporting
 OID:1.3.6.1.4.1.25623.1.0.105937
 Version used: $Revision: 14244 $</t>
-        </is>
-      </c>
-      <c r="Q34" t="inlineStr"/>
-      <c r="R34" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S34" t="inlineStr">
-        <is>
-          <t>[]</t>
         </is>
       </c>
     </row>
@@ -3003,14 +2417,11 @@
           <t>Block unwanted packets from escaping your network.</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
           <t>LOG</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
           <t>general</t>
@@ -3029,30 +2440,16 @@
       <c r="K35" t="n">
         <v>0</v>
       </c>
-      <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr">
         <is>
           <t>Here is the route from 127.0.0.1 to 127.0.0.1: 127.0.0.1</t>
         </is>
       </c>
-      <c r="N35" t="inlineStr"/>
-      <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr">
         <is>
           <t>Details: Traceroute
 OID:1.3.6.1.4.1.25623.1.0.51662
 Version used: $Revision: 10411 $</t>
-        </is>
-      </c>
-      <c r="Q35" t="inlineStr"/>
-      <c r="R35" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="S35" t="inlineStr">
-        <is>
-          <t>[]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
resources: restore dropped ligatures in the OpenVAS baselines
The PDF export lost ff/fi/fl ligatures (certificate -> certicate,
Diffie-Hellman -> Die-Hellman), so correct extractions were scored as
wrong. 55 words across 48 cells, plus 3 cells where the ligature was
escaped as _x001E_/_x001F_/_x0011_. Corrections come from the reader,
which restores them, and preserve the original casing.
</commit_message>
<xml_diff>
--- a/resources/openvas/OpenVAS_JuiceShop.xlsx
+++ b/resources/openvas/OpenVAS_JuiceShop.xlsx
@@ -554,7 +554,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>The remote OpenVAS / Greenbone Vulnerability Manager is installed/congured in a way that it has account(s) with default passwords enabled.</t>
+          <t>The remote OpenVAS / Greenbone Vulnerability Manager is installed/configured in a way that it has account(s) with default passwords enabled.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -622,7 +622,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Replace the SSL/TLS certicate by a new one.</t>
+          <t>Replace the SSL/TLS certificate by a new one.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -648,7 +648,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>This script checks expiry dates of certicates associated with SSL/TLS-enabled services on the target and reports whether any have already expired.</t>
+          <t>This script checks expiry dates of certificates associated with SSL/TLS-enabled services on the target and reports whether any have already expired.</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -745,7 +745,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Replace the SSL/TLS certicate by a new one.</t>
+          <t>Replace the SSL/TLS certificate by a new one.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -771,7 +771,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>This script checks expiry dates of certicates associated with SSL/TLS-enabled services on the target and reports whether any have already expired.</t>
+          <t>This script checks expiry dates of certificates associated with SSL/TLS-enabled services on the target and reports whether any have already expired.</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1088,7 +1088,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>This script collects and reports the details of all SSL/TLS certicates.</t>
+          <t>This script collects and reports the details of all SSL/TLS certificates.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1148,7 +1148,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>['Enable HPKP or add / congure the required directives correctly following the guides linked in the references.']</t>
+          <t>['Enable HPKP or add / configure the required directives correctly following the guides linked in the references.']</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1212,7 +1212,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Enable HSTS or add / congure the required directives correctly following the guides linked in the references.</t>
+          <t>Enable HSTS or add / configure the required directives correctly following the guides linked in the references.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1556,7 +1556,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>The script checks the SMTP server banner for the presence of Postx.</t>
+          <t>The script checks the SMTP server banner for the presence of Postfix.</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">

</xml_diff>